<commit_message>
P02b: calibrate baseline motor third-party liability premium
Premium per policy 5,500 to 9,500; ten-year gross ultimate loss ratio 1.77 to 1.03.
Other lines were inside their ranges. Fixtures and examples regenerated.
Records 0018 (new) and 0017 (CV07 1.1.0 allows title rows).
</commit_message>
<xml_diff>
--- a/examples/baseline/expenses.xlsx
+++ b/examples/baseline/expenses.xlsx
@@ -422,7 +422,7 @@
         <v>44592</v>
       </c>
       <c r="B3">
-        <v>2042.35</v>
+        <v>3527.7</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -521,7 +521,7 @@
         <v>44592</v>
       </c>
       <c r="B6">
-        <v>2189.1</v>
+        <v>3781.18</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -620,7 +620,7 @@
         <v>44592</v>
       </c>
       <c r="B9">
-        <v>9530.98</v>
+        <v>16462.61</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -719,7 +719,7 @@
         <v>44592</v>
       </c>
       <c r="B12">
-        <v>10215.81</v>
+        <v>17645.5</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -785,7 +785,7 @@
         <v>44592</v>
       </c>
       <c r="B14">
-        <v>2488.8</v>
+        <v>3479.03</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -808,7 +808,7 @@
         <v>44592</v>
       </c>
       <c r="B15">
-        <v>2216.19</v>
+        <v>3277.57</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -887,7 +887,7 @@
         <v>44620</v>
       </c>
       <c r="B18">
-        <v>1944.01</v>
+        <v>3357.84</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
         <v>44620</v>
       </c>
       <c r="B21">
-        <v>1998.73</v>
+        <v>3452.35</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         <v>44620</v>
       </c>
       <c r="B24">
-        <v>9072.059999999999</v>
+        <v>15669.92</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1184,7 +1184,7 @@
         <v>44620</v>
       </c>
       <c r="B27">
-        <v>9327.4</v>
+        <v>16110.96</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1250,7 +1250,7 @@
         <v>44620</v>
       </c>
       <c r="B29">
-        <v>2377.88</v>
+        <v>3320.43</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
         <v>44620</v>
       </c>
       <c r="B30">
-        <v>2033.24</v>
+        <v>3002.32</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1352,7 +1352,7 @@
         <v>44651</v>
       </c>
       <c r="B33">
-        <v>2334.71</v>
+        <v>4032.68</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1451,7 +1451,7 @@
         <v>44651</v>
       </c>
       <c r="B36">
-        <v>2309.51</v>
+        <v>3989.16</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1550,7 +1550,7 @@
         <v>44651</v>
       </c>
       <c r="B39">
-        <v>10895.3</v>
+        <v>18819.16</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1649,7 +1649,7 @@
         <v>44651</v>
       </c>
       <c r="B42">
-        <v>10777.72</v>
+        <v>18616.07</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1814,7 +1814,7 @@
         <v>44651</v>
       </c>
       <c r="B47">
-        <v>2832.12</v>
+        <v>3964.1</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
         <v>44651</v>
       </c>
       <c r="B48">
-        <v>2345.25</v>
+        <v>3465.01</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1916,7 +1916,7 @@
         <v>44681</v>
       </c>
       <c r="B51">
-        <v>2381.99</v>
+        <v>4114.34</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -2015,7 +2015,7 @@
         <v>44681</v>
       </c>
       <c r="B54">
-        <v>2329.63</v>
+        <v>4023.91</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -2114,7 +2114,7 @@
         <v>44681</v>
       </c>
       <c r="B57">
-        <v>11115.94</v>
+        <v>19200.26</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -2213,7 +2213,7 @@
         <v>44681</v>
       </c>
       <c r="B60">
-        <v>10871.62</v>
+        <v>18778.25</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -2312,7 +2312,7 @@
         <v>44681</v>
       </c>
       <c r="B63">
-        <v>2933.22</v>
+        <v>4088.12</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -2335,7 +2335,7 @@
         <v>44681</v>
       </c>
       <c r="B64">
-        <v>2365.14</v>
+        <v>3494.66</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -2414,7 +2414,7 @@
         <v>44712</v>
       </c>
       <c r="B67">
-        <v>2551.1</v>
+        <v>4406.45</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -2513,7 +2513,7 @@
         <v>44712</v>
       </c>
       <c r="B70">
-        <v>2528.67</v>
+        <v>4367.71</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2612,7 +2612,7 @@
         <v>44712</v>
       </c>
       <c r="B73">
-        <v>11905.15</v>
+        <v>20563.44</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
         <v>44712</v>
       </c>
       <c r="B76">
-        <v>11800.47</v>
+        <v>20382.63</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2843,7 +2843,7 @@
         <v>44712</v>
       </c>
       <c r="B80">
-        <v>3101.66</v>
+        <v>4338.56</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2866,7 +2866,7 @@
         <v>44712</v>
       </c>
       <c r="B81">
-        <v>2617.3</v>
+        <v>3843.32</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2945,7 +2945,7 @@
         <v>44742</v>
       </c>
       <c r="B84">
-        <v>2538.63</v>
+        <v>4384.9</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -3044,7 +3044,7 @@
         <v>44742</v>
       </c>
       <c r="B87">
-        <v>2628.81</v>
+        <v>4540.68</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -3143,7 +3143,7 @@
         <v>44742</v>
       </c>
       <c r="B90">
-        <v>11846.93</v>
+        <v>20462.87</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -3242,7 +3242,7 @@
         <v>44742</v>
       </c>
       <c r="B93">
-        <v>12267.8</v>
+        <v>21189.84</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -3407,7 +3407,7 @@
         <v>44742</v>
       </c>
       <c r="B98">
-        <v>3076.13</v>
+        <v>4306.98</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -3430,7 +3430,7 @@
         <v>44742</v>
       </c>
       <c r="B99">
-        <v>2717.04</v>
+        <v>3991.62</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -3509,7 +3509,7 @@
         <v>44773</v>
       </c>
       <c r="B102">
-        <v>2664.47</v>
+        <v>4602.27</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
@@ -3608,7 +3608,7 @@
         <v>44773</v>
       </c>
       <c r="B105">
-        <v>2782.93</v>
+        <v>4806.88</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -3707,7 +3707,7 @@
         <v>44773</v>
       </c>
       <c r="B108">
-        <v>12434.19</v>
+        <v>21477.24</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
@@ -3806,7 +3806,7 @@
         <v>44773</v>
       </c>
       <c r="B111">
-        <v>12987.01</v>
+        <v>22432.11</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -4004,7 +4004,7 @@
         <v>44773</v>
       </c>
       <c r="B117">
-        <v>3250.8</v>
+        <v>4542.66</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
@@ -4027,7 +4027,7 @@
         <v>44773</v>
       </c>
       <c r="B118">
-        <v>2919.86</v>
+        <v>4269.16</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
@@ -4106,7 +4106,7 @@
         <v>44804</v>
       </c>
       <c r="B121">
-        <v>2855.92</v>
+        <v>4932.96</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
@@ -4205,7 +4205,7 @@
         <v>44804</v>
       </c>
       <c r="B124">
-        <v>2871.03</v>
+        <v>4959.04</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
@@ -4304,7 +4304,7 @@
         <v>44804</v>
       </c>
       <c r="B127">
-        <v>13327.64</v>
+        <v>23020.48</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
@@ -4403,7 +4403,7 @@
         <v>44804</v>
       </c>
       <c r="B130">
-        <v>13398.12</v>
+        <v>23142.21</v>
       </c>
       <c r="C130" t="inlineStr">
         <is>
@@ -4568,7 +4568,7 @@
         <v>44804</v>
       </c>
       <c r="B135">
-        <v>3350.72</v>
+        <v>4735.41</v>
       </c>
       <c r="C135" t="inlineStr">
         <is>
@@ -4591,7 +4591,7 @@
         <v>44804</v>
       </c>
       <c r="B136">
-        <v>3014.47</v>
+        <v>4406.49</v>
       </c>
       <c r="C136" t="inlineStr">
         <is>
@@ -4670,7 +4670,7 @@
         <v>44834</v>
       </c>
       <c r="B139">
-        <v>2774.66</v>
+        <v>4792.6</v>
       </c>
       <c r="C139" t="inlineStr">
         <is>
@@ -4769,7 +4769,7 @@
         <v>44834</v>
       </c>
       <c r="B142">
-        <v>2831.55</v>
+        <v>4890.86</v>
       </c>
       <c r="C142" t="inlineStr">
         <is>
@@ -4868,7 +4868,7 @@
         <v>44834</v>
       </c>
       <c r="B145">
-        <v>12948.43</v>
+        <v>22365.47</v>
       </c>
       <c r="C145" t="inlineStr">
         <is>
@@ -4967,7 +4967,7 @@
         <v>44834</v>
       </c>
       <c r="B148">
-        <v>13213.9</v>
+        <v>22824.02</v>
       </c>
       <c r="C148" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
         <v>44834</v>
       </c>
       <c r="B155">
-        <v>3321.62</v>
+        <v>4666.91</v>
       </c>
       <c r="C155" t="inlineStr">
         <is>
@@ -5221,7 +5221,7 @@
         <v>44834</v>
       </c>
       <c r="B156">
-        <v>3025.84</v>
+        <v>4398.72</v>
       </c>
       <c r="C156" t="inlineStr">
         <is>
@@ -5300,7 +5300,7 @@
         <v>44865</v>
       </c>
       <c r="B159">
-        <v>3058.2</v>
+        <v>5282.34</v>
       </c>
       <c r="C159" t="inlineStr">
         <is>
@@ -5399,7 +5399,7 @@
         <v>44865</v>
       </c>
       <c r="B162">
-        <v>3165.29</v>
+        <v>5467.31</v>
       </c>
       <c r="C162" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
         <v>44865</v>
       </c>
       <c r="B165">
-        <v>14271.6</v>
+        <v>24650.94</v>
       </c>
       <c r="C165" t="inlineStr">
         <is>
@@ -5597,7 +5597,7 @@
         <v>44865</v>
       </c>
       <c r="B168">
-        <v>14771.34</v>
+        <v>25514.13</v>
       </c>
       <c r="C168" t="inlineStr">
         <is>
@@ -5729,7 +5729,7 @@
         <v>44865</v>
       </c>
       <c r="B172">
-        <v>3572.53</v>
+        <v>5055.3</v>
       </c>
       <c r="C172" t="inlineStr">
         <is>
@@ -5752,7 +5752,7 @@
         <v>44865</v>
       </c>
       <c r="B173">
-        <v>3311.08</v>
+        <v>4845.77</v>
       </c>
       <c r="C173" t="inlineStr">
         <is>
@@ -5831,7 +5831,7 @@
         <v>44895</v>
       </c>
       <c r="B176">
-        <v>3033.34</v>
+        <v>5239.41</v>
       </c>
       <c r="C176" t="inlineStr">
         <is>
@@ -5930,7 +5930,7 @@
         <v>44895</v>
       </c>
       <c r="B179">
-        <v>3195.13</v>
+        <v>5518.86</v>
       </c>
       <c r="C179" t="inlineStr">
         <is>
@@ -6029,7 +6029,7 @@
         <v>44895</v>
       </c>
       <c r="B182">
-        <v>14155.6</v>
+        <v>24450.59</v>
       </c>
       <c r="C182" t="inlineStr">
         <is>
@@ -6128,7 +6128,7 @@
         <v>44895</v>
       </c>
       <c r="B185">
-        <v>14910.61</v>
+        <v>25754.69</v>
       </c>
       <c r="C185" t="inlineStr">
         <is>
@@ -6260,7 +6260,7 @@
         <v>44895</v>
       </c>
       <c r="B189">
-        <v>3590.08</v>
+        <v>5060.8</v>
       </c>
       <c r="C189" t="inlineStr">
         <is>
@@ -6283,7 +6283,7 @@
         <v>44895</v>
       </c>
       <c r="B190">
-        <v>3414.92</v>
+        <v>4964.08</v>
       </c>
       <c r="C190" t="inlineStr">
         <is>
@@ -6362,7 +6362,7 @@
         <v>44926</v>
       </c>
       <c r="B193">
-        <v>3221.69</v>
+        <v>5564.73</v>
       </c>
       <c r="C193" t="inlineStr">
         <is>
@@ -6461,7 +6461,7 @@
         <v>44926</v>
       </c>
       <c r="B196">
-        <v>3296.98</v>
+        <v>5694.79</v>
       </c>
       <c r="C196" t="inlineStr">
         <is>
@@ -6560,7 +6560,7 @@
         <v>44926</v>
       </c>
       <c r="B199">
-        <v>15034.53</v>
+        <v>25968.74</v>
       </c>
       <c r="C199" t="inlineStr">
         <is>
@@ -6659,7 +6659,7 @@
         <v>44926</v>
       </c>
       <c r="B202">
-        <v>15385.92</v>
+        <v>26575.68</v>
       </c>
       <c r="C202" t="inlineStr">
         <is>
@@ -6857,7 +6857,7 @@
         <v>44926</v>
       </c>
       <c r="B208">
-        <v>3837.68</v>
+        <v>5399.71</v>
       </c>
       <c r="C208" t="inlineStr">
         <is>
@@ -6880,7 +6880,7 @@
         <v>44926</v>
       </c>
       <c r="B209">
-        <v>3684.21</v>
+        <v>5282.75</v>
       </c>
       <c r="C209" t="inlineStr">
         <is>
@@ -6959,7 +6959,7 @@
         <v>44957</v>
       </c>
       <c r="B212">
-        <v>3297.34</v>
+        <v>5695.41</v>
       </c>
       <c r="C212" t="inlineStr">
         <is>
@@ -7058,7 +7058,7 @@
         <v>44957</v>
       </c>
       <c r="B215">
-        <v>3422.45</v>
+        <v>5911.5</v>
       </c>
       <c r="C215" t="inlineStr">
         <is>
@@ -7157,7 +7157,7 @@
         <v>44957</v>
       </c>
       <c r="B218">
-        <v>15387.59</v>
+        <v>26578.57</v>
       </c>
       <c r="C218" t="inlineStr">
         <is>
@@ -7256,7 +7256,7 @@
         <v>44957</v>
       </c>
       <c r="B221">
-        <v>15971.41</v>
+        <v>27586.99</v>
       </c>
       <c r="C221" t="inlineStr">
         <is>
@@ -7421,7 +7421,7 @@
         <v>44957</v>
       </c>
       <c r="B226">
-        <v>3816.33</v>
+        <v>5415.04</v>
       </c>
       <c r="C226" t="inlineStr">
         <is>
@@ -7444,7 +7444,7 @@
         <v>44957</v>
       </c>
       <c r="B227">
-        <v>3774.28</v>
+        <v>5433.64</v>
       </c>
       <c r="C227" t="inlineStr">
         <is>
@@ -7523,7 +7523,7 @@
         <v>44985</v>
       </c>
       <c r="B230">
-        <v>2957.93</v>
+        <v>5109.15</v>
       </c>
       <c r="C230" t="inlineStr">
         <is>
@@ -7622,7 +7622,7 @@
         <v>44985</v>
       </c>
       <c r="B233">
-        <v>3321.42</v>
+        <v>5737</v>
       </c>
       <c r="C233" t="inlineStr">
         <is>
@@ -7721,7 +7721,7 @@
         <v>44985</v>
       </c>
       <c r="B236">
-        <v>13803.68</v>
+        <v>23842.72</v>
       </c>
       <c r="C236" t="inlineStr">
         <is>
@@ -7820,7 +7820,7 @@
         <v>44985</v>
       </c>
       <c r="B239">
-        <v>15499.96</v>
+        <v>26772.65</v>
       </c>
       <c r="C239" t="inlineStr">
         <is>
@@ -7952,7 +7952,7 @@
         <v>44985</v>
       </c>
       <c r="B243">
-        <v>3456.26</v>
+        <v>4890.41</v>
       </c>
       <c r="C243" t="inlineStr">
         <is>
@@ -7975,7 +7975,7 @@
         <v>44985</v>
       </c>
       <c r="B244">
-        <v>3671.22</v>
+        <v>5281.6</v>
       </c>
       <c r="C244" t="inlineStr">
         <is>
@@ -8054,7 +8054,7 @@
         <v>45016</v>
       </c>
       <c r="B247">
-        <v>3449.41</v>
+        <v>5958.07</v>
       </c>
       <c r="C247" t="inlineStr">
         <is>
@@ -8153,7 +8153,7 @@
         <v>45016</v>
       </c>
       <c r="B250">
-        <v>3760.65</v>
+        <v>6495.67</v>
       </c>
       <c r="C250" t="inlineStr">
         <is>
@@ -8252,7 +8252,7 @@
         <v>45016</v>
       </c>
       <c r="B253">
-        <v>16097.24</v>
+        <v>27804.33</v>
       </c>
       <c r="C253" t="inlineStr">
         <is>
@@ -8351,7 +8351,7 @@
         <v>45016</v>
       </c>
       <c r="B256">
-        <v>17549.71</v>
+        <v>30313.14</v>
       </c>
       <c r="C256" t="inlineStr">
         <is>
@@ -8483,7 +8483,7 @@
         <v>45016</v>
       </c>
       <c r="B260">
-        <v>4099.67</v>
+        <v>5772.11</v>
       </c>
       <c r="C260" t="inlineStr">
         <is>
@@ -8506,7 +8506,7 @@
         <v>45016</v>
       </c>
       <c r="B261">
-        <v>4269.88</v>
+        <v>6093.23</v>
       </c>
       <c r="C261" t="inlineStr">
         <is>
@@ -8585,7 +8585,7 @@
         <v>45046</v>
       </c>
       <c r="B264">
-        <v>3513.37</v>
+        <v>6068.56</v>
       </c>
       <c r="C264" t="inlineStr">
         <is>
@@ -8684,7 +8684,7 @@
         <v>45046</v>
       </c>
       <c r="B267">
-        <v>3793.47</v>
+        <v>6552.35</v>
       </c>
       <c r="C267" t="inlineStr">
         <is>
@@ -8783,7 +8783,7 @@
         <v>45046</v>
       </c>
       <c r="B270">
-        <v>16395.75</v>
+        <v>28319.93</v>
       </c>
       <c r="C270" t="inlineStr">
         <is>
@@ -8882,7 +8882,7 @@
         <v>45046</v>
       </c>
       <c r="B273">
-        <v>17702.84</v>
+        <v>30577.64</v>
       </c>
       <c r="C273" t="inlineStr">
         <is>
@@ -9014,7 +9014,7 @@
         <v>45046</v>
       </c>
       <c r="B277">
-        <v>4399.8</v>
+        <v>6103.26</v>
       </c>
       <c r="C277" t="inlineStr">
         <is>
@@ -9037,7 +9037,7 @@
         <v>45046</v>
       </c>
       <c r="B278">
-        <v>4231.54</v>
+        <v>6070.8</v>
       </c>
       <c r="C278" t="inlineStr">
         <is>
@@ -9116,7 +9116,7 @@
         <v>45077</v>
       </c>
       <c r="B281">
-        <v>3886.2</v>
+        <v>6712.53</v>
       </c>
       <c r="C281" t="inlineStr">
         <is>
@@ -9215,7 +9215,7 @@
         <v>45077</v>
       </c>
       <c r="B284">
-        <v>4186.14</v>
+        <v>7230.6</v>
       </c>
       <c r="C284" t="inlineStr">
         <is>
@@ -9314,7 +9314,7 @@
         <v>45077</v>
       </c>
       <c r="B287">
-        <v>18135.6</v>
+        <v>31325.13</v>
       </c>
       <c r="C287" t="inlineStr">
         <is>
@@ -9413,7 +9413,7 @@
         <v>45077</v>
       </c>
       <c r="B290">
-        <v>19535.31</v>
+        <v>33742.81</v>
       </c>
       <c r="C290" t="inlineStr">
         <is>
@@ -9611,7 +9611,7 @@
         <v>45077</v>
       </c>
       <c r="B296">
-        <v>4974.52</v>
+        <v>6858.74</v>
       </c>
       <c r="C296" t="inlineStr">
         <is>
@@ -9634,7 +9634,7 @@
         <v>45077</v>
       </c>
       <c r="B297">
-        <v>4571.3</v>
+        <v>6600.94</v>
       </c>
       <c r="C297" t="inlineStr">
         <is>
@@ -9713,7 +9713,7 @@
         <v>45107</v>
       </c>
       <c r="B300">
-        <v>3930.18</v>
+        <v>6788.5</v>
       </c>
       <c r="C300" t="inlineStr">
         <is>
@@ -9812,7 +9812,7 @@
         <v>45107</v>
       </c>
       <c r="B303">
-        <v>4464.32</v>
+        <v>7711.1</v>
       </c>
       <c r="C303" t="inlineStr">
         <is>
@@ -9911,7 +9911,7 @@
         <v>45107</v>
       </c>
       <c r="B306">
-        <v>18340.86</v>
+        <v>31679.67</v>
       </c>
       <c r="C306" t="inlineStr">
         <is>
@@ -10010,7 +10010,7 @@
         <v>45107</v>
       </c>
       <c r="B309">
-        <v>20833.5</v>
+        <v>35985.13</v>
       </c>
       <c r="C309" t="inlineStr">
         <is>
@@ -10208,7 +10208,7 @@
         <v>45107</v>
       </c>
       <c r="B315">
-        <v>5100.6</v>
+        <v>7006.14</v>
       </c>
       <c r="C315" t="inlineStr">
         <is>
@@ -10231,7 +10231,7 @@
         <v>45107</v>
       </c>
       <c r="B316">
-        <v>4718.82</v>
+        <v>6883.34</v>
       </c>
       <c r="C316" t="inlineStr">
         <is>
@@ -10310,7 +10310,7 @@
         <v>45138</v>
       </c>
       <c r="B319">
-        <v>4260.83</v>
+        <v>7359.61</v>
       </c>
       <c r="C319" t="inlineStr">
         <is>
@@ -10409,7 +10409,7 @@
         <v>45138</v>
       </c>
       <c r="B322">
-        <v>4744.59</v>
+        <v>8195.200000000001</v>
       </c>
       <c r="C322" t="inlineStr">
         <is>
@@ -10508,7 +10508,7 @@
         <v>45138</v>
       </c>
       <c r="B325">
-        <v>19883.86</v>
+        <v>34344.85</v>
       </c>
       <c r="C325" t="inlineStr">
         <is>
@@ -10607,7 +10607,7 @@
         <v>45138</v>
       </c>
       <c r="B328">
-        <v>22141.41</v>
+        <v>38244.26</v>
       </c>
       <c r="C328" t="inlineStr">
         <is>
@@ -10838,7 +10838,7 @@
         <v>45138</v>
       </c>
       <c r="B335">
-        <v>5424.8</v>
+        <v>7490.65</v>
       </c>
       <c r="C335" t="inlineStr">
         <is>
@@ -10861,7 +10861,7 @@
         <v>45138</v>
       </c>
       <c r="B336">
-        <v>5216.61</v>
+        <v>7517.01</v>
       </c>
       <c r="C336" t="inlineStr">
         <is>
@@ -10940,7 +10940,7 @@
         <v>45169</v>
       </c>
       <c r="B339">
-        <v>4539.27</v>
+        <v>7840.55</v>
       </c>
       <c r="C339" t="inlineStr">
         <is>
@@ -11039,7 +11039,7 @@
         <v>45169</v>
       </c>
       <c r="B342">
-        <v>4845.72</v>
+        <v>8369.879999999999</v>
       </c>
       <c r="C342" t="inlineStr">
         <is>
@@ -11138,7 +11138,7 @@
         <v>45169</v>
       </c>
       <c r="B345">
-        <v>21183.24</v>
+        <v>36589.24</v>
       </c>
       <c r="C345" t="inlineStr">
         <is>
@@ -11237,7 +11237,7 @@
         <v>45169</v>
       </c>
       <c r="B348">
-        <v>22613.35</v>
+        <v>39059.42</v>
       </c>
       <c r="C348" t="inlineStr">
         <is>
@@ -11402,7 +11402,7 @@
         <v>45169</v>
       </c>
       <c r="B353">
-        <v>5919.99</v>
+        <v>8120.85</v>
       </c>
       <c r="C353" t="inlineStr">
         <is>
@@ -11425,7 +11425,7 @@
         <v>45169</v>
       </c>
       <c r="B354">
-        <v>5273.51</v>
+        <v>7622.95</v>
       </c>
       <c r="C354" t="inlineStr">
         <is>
@@ -11504,7 +11504,7 @@
         <v>45199</v>
       </c>
       <c r="B357">
-        <v>4533.28</v>
+        <v>7830.22</v>
       </c>
       <c r="C357" t="inlineStr">
         <is>
@@ -11603,7 +11603,7 @@
         <v>45199</v>
       </c>
       <c r="B360">
-        <v>4773.06</v>
+        <v>8244.379999999999</v>
       </c>
       <c r="C360" t="inlineStr">
         <is>
@@ -11702,7 +11702,7 @@
         <v>45199</v>
       </c>
       <c r="B363">
-        <v>21155.32</v>
+        <v>36541.01</v>
       </c>
       <c r="C363" t="inlineStr">
         <is>
@@ -11801,7 +11801,7 @@
         <v>45199</v>
       </c>
       <c r="B366">
-        <v>22274.3</v>
+        <v>38473.79</v>
       </c>
       <c r="C366" t="inlineStr">
         <is>
@@ -11966,7 +11966,7 @@
         <v>45199</v>
       </c>
       <c r="B371">
-        <v>6053.92</v>
+        <v>8251.879999999999</v>
       </c>
       <c r="C371" t="inlineStr">
         <is>
@@ -11989,7 +11989,7 @@
         <v>45199</v>
       </c>
       <c r="B372">
-        <v>5112.39</v>
+        <v>7426.6</v>
       </c>
       <c r="C372" t="inlineStr">
         <is>
@@ -12068,7 +12068,7 @@
         <v>45230</v>
       </c>
       <c r="B375">
-        <v>4680.38</v>
+        <v>8084.3</v>
       </c>
       <c r="C375" t="inlineStr">
         <is>
@@ -12167,7 +12167,7 @@
         <v>45230</v>
       </c>
       <c r="B378">
-        <v>4842.14</v>
+        <v>8363.700000000001</v>
       </c>
       <c r="C378" t="inlineStr">
         <is>
@@ -12266,7 +12266,7 @@
         <v>45230</v>
       </c>
       <c r="B381">
-        <v>21841.78</v>
+        <v>37726.71</v>
       </c>
       <c r="C381" t="inlineStr">
         <is>
@@ -12365,7 +12365,7 @@
         <v>45230</v>
       </c>
       <c r="B384">
-        <v>22596.65</v>
+        <v>39030.58</v>
       </c>
       <c r="C384" t="inlineStr">
         <is>
@@ -12563,7 +12563,7 @@
         <v>45230</v>
       </c>
       <c r="B390">
-        <v>6353.77</v>
+        <v>8623.049999999999</v>
       </c>
       <c r="C390" t="inlineStr">
         <is>
@@ -12586,7 +12586,7 @@
         <v>45230</v>
       </c>
       <c r="B391">
-        <v>5225.4</v>
+        <v>7573.1</v>
       </c>
       <c r="C391" t="inlineStr">
         <is>
@@ -12665,7 +12665,7 @@
         <v>45260</v>
       </c>
       <c r="B394">
-        <v>4771.1</v>
+        <v>8240.98</v>
       </c>
       <c r="C394" t="inlineStr">
         <is>
@@ -12764,7 +12764,7 @@
         <v>45260</v>
       </c>
       <c r="B397">
-        <v>4913.42</v>
+        <v>8486.809999999999</v>
       </c>
       <c r="C397" t="inlineStr">
         <is>
@@ -12863,7 +12863,7 @@
         <v>45260</v>
       </c>
       <c r="B400">
-        <v>22265.11</v>
+        <v>38457.92</v>
       </c>
       <c r="C400" t="inlineStr">
         <is>
@@ -12962,7 +12962,7 @@
         <v>45260</v>
       </c>
       <c r="B403">
-        <v>22929.28</v>
+        <v>39605.12</v>
       </c>
       <c r="C403" t="inlineStr">
         <is>
@@ -13127,7 +13127,7 @@
         <v>45260</v>
       </c>
       <c r="B408">
-        <v>6337.67</v>
+        <v>8650.93</v>
       </c>
       <c r="C408" t="inlineStr">
         <is>
@@ -13150,7 +13150,7 @@
         <v>45260</v>
       </c>
       <c r="B409">
-        <v>5150.21</v>
+        <v>7532.47</v>
       </c>
       <c r="C409" t="inlineStr">
         <is>
@@ -13229,7 +13229,7 @@
         <v>45291</v>
       </c>
       <c r="B412">
-        <v>5247.58</v>
+        <v>9064</v>
       </c>
       <c r="C412" t="inlineStr">
         <is>
@@ -13328,7 +13328,7 @@
         <v>45291</v>
       </c>
       <c r="B415">
-        <v>5405.62</v>
+        <v>9336.99</v>
       </c>
       <c r="C415" t="inlineStr">
         <is>
@@ -13427,7 +13427,7 @@
         <v>45291</v>
       </c>
       <c r="B418">
-        <v>24488.71</v>
+        <v>42298.68</v>
       </c>
       <c r="C418" t="inlineStr">
         <is>
@@ -13526,7 +13526,7 @@
         <v>45291</v>
       </c>
       <c r="B421">
-        <v>25226.25</v>
+        <v>43572.61</v>
       </c>
       <c r="C421" t="inlineStr">
         <is>
@@ -13658,7 +13658,7 @@
         <v>45291</v>
       </c>
       <c r="B425">
-        <v>6697.85</v>
+        <v>9242.139999999999</v>
       </c>
       <c r="C425" t="inlineStr">
         <is>
@@ -13681,7 +13681,7 @@
         <v>45291</v>
       </c>
       <c r="B426">
-        <v>5534.58</v>
+        <v>8155.49</v>
       </c>
       <c r="C426" t="inlineStr">
         <is>
@@ -13760,7 +13760,7 @@
         <v>45322</v>
       </c>
       <c r="B429">
-        <v>5535.05</v>
+        <v>9560.540000000001</v>
       </c>
       <c r="C429" t="inlineStr">
         <is>
@@ -13859,7 +13859,7 @@
         <v>45322</v>
       </c>
       <c r="B432">
-        <v>5617.85</v>
+        <v>9703.559999999999</v>
       </c>
       <c r="C432" t="inlineStr">
         <is>
@@ -13958,7 +13958,7 @@
         <v>45322</v>
       </c>
       <c r="B435">
-        <v>25830.23</v>
+        <v>44615.85</v>
       </c>
       <c r="C435" t="inlineStr">
         <is>
@@ -14057,7 +14057,7 @@
         <v>45322</v>
       </c>
       <c r="B438">
-        <v>26216.64</v>
+        <v>45283.29</v>
       </c>
       <c r="C438" t="inlineStr">
         <is>
@@ -14222,7 +14222,7 @@
         <v>45322</v>
       </c>
       <c r="B443">
-        <v>6996.24</v>
+        <v>9679.9</v>
       </c>
       <c r="C443" t="inlineStr">
         <is>
@@ -14245,7 +14245,7 @@
         <v>45322</v>
       </c>
       <c r="B444">
-        <v>5745.14</v>
+        <v>8468.950000000001</v>
       </c>
       <c r="C444" t="inlineStr">
         <is>
@@ -14324,7 +14324,7 @@
         <v>45351</v>
       </c>
       <c r="B447">
-        <v>5541.04</v>
+        <v>9570.889999999999</v>
       </c>
       <c r="C447" t="inlineStr">
         <is>
@@ -14423,7 +14423,7 @@
         <v>45351</v>
       </c>
       <c r="B450">
-        <v>5575</v>
+        <v>9629.549999999999</v>
       </c>
       <c r="C450" t="inlineStr">
         <is>
@@ -14522,7 +14522,7 @@
         <v>45351</v>
       </c>
       <c r="B453">
-        <v>25858.2</v>
+        <v>44664.17</v>
       </c>
       <c r="C453" t="inlineStr">
         <is>
@@ -14621,7 +14621,7 @@
         <v>45351</v>
       </c>
       <c r="B456">
-        <v>26016.67</v>
+        <v>44937.88</v>
       </c>
       <c r="C456" t="inlineStr">
         <is>
@@ -14753,7 +14753,7 @@
         <v>45351</v>
       </c>
       <c r="B460">
-        <v>7038.6</v>
+        <v>9725.16</v>
       </c>
       <c r="C460" t="inlineStr">
         <is>
@@ -14776,7 +14776,7 @@
         <v>45351</v>
       </c>
       <c r="B461">
-        <v>5631.63</v>
+        <v>8334.66</v>
       </c>
       <c r="C461" t="inlineStr">
         <is>
@@ -14855,7 +14855,7 @@
         <v>45382</v>
       </c>
       <c r="B464">
-        <v>6336.53</v>
+        <v>10944.92</v>
       </c>
       <c r="C464" t="inlineStr">
         <is>
@@ -14954,7 +14954,7 @@
         <v>45382</v>
       </c>
       <c r="B467">
-        <v>6219.87</v>
+        <v>10743.42</v>
       </c>
       <c r="C467" t="inlineStr">
         <is>
@@ -15053,7 +15053,7 @@
         <v>45382</v>
       </c>
       <c r="B470">
-        <v>29570.49</v>
+        <v>51076.3</v>
       </c>
       <c r="C470" t="inlineStr">
         <is>
@@ -15152,7 +15152,7 @@
         <v>45382</v>
       </c>
       <c r="B473">
-        <v>29026.08</v>
+        <v>50135.96</v>
       </c>
       <c r="C473" t="inlineStr">
         <is>
@@ -15284,7 +15284,7 @@
         <v>45382</v>
       </c>
       <c r="B477">
-        <v>7596.25</v>
+        <v>10668.51</v>
       </c>
       <c r="C477" t="inlineStr">
         <is>
@@ -15307,7 +15307,7 @@
         <v>45382</v>
       </c>
       <c r="B478">
-        <v>6278.01</v>
+        <v>9293.709999999999</v>
       </c>
       <c r="C478" t="inlineStr">
         <is>
@@ -15386,7 +15386,7 @@
         <v>45412</v>
       </c>
       <c r="B481">
-        <v>6183.12</v>
+        <v>10679.93</v>
       </c>
       <c r="C481" t="inlineStr">
         <is>
@@ -15485,7 +15485,7 @@
         <v>45412</v>
       </c>
       <c r="B484">
-        <v>6444.72</v>
+        <v>11131.79</v>
       </c>
       <c r="C484" t="inlineStr">
         <is>
@@ -15584,7 +15584,7 @@
         <v>45412</v>
       </c>
       <c r="B487">
-        <v>28854.55</v>
+        <v>49839.67</v>
       </c>
       <c r="C487" t="inlineStr">
         <is>
@@ -15683,7 +15683,7 @@
         <v>45412</v>
       </c>
       <c r="B490">
-        <v>30075.37</v>
+        <v>51948.36</v>
       </c>
       <c r="C490" t="inlineStr">
         <is>
@@ -15815,7 +15815,7 @@
         <v>45412</v>
       </c>
       <c r="B494">
-        <v>7136.05</v>
+        <v>10133.92</v>
       </c>
       <c r="C494" t="inlineStr">
         <is>
@@ -15838,7 +15838,7 @@
         <v>45412</v>
       </c>
       <c r="B495">
-        <v>6449.06</v>
+        <v>9573.780000000001</v>
       </c>
       <c r="C495" t="inlineStr">
         <is>
@@ -15917,7 +15917,7 @@
         <v>45443</v>
       </c>
       <c r="B498">
-        <v>6402.52</v>
+        <v>11058.9</v>
       </c>
       <c r="C498" t="inlineStr">
         <is>
@@ -16016,7 +16016,7 @@
         <v>45443</v>
       </c>
       <c r="B501">
-        <v>7000.73</v>
+        <v>12092.17</v>
       </c>
       <c r="C501" t="inlineStr">
         <is>
@@ -16115,7 +16115,7 @@
         <v>45443</v>
       </c>
       <c r="B504">
-        <v>29878.44</v>
+        <v>51608.22</v>
       </c>
       <c r="C504" t="inlineStr">
         <is>
@@ -16214,7 +16214,7 @@
         <v>45443</v>
       </c>
       <c r="B507">
-        <v>32670.08</v>
+        <v>56430.13</v>
       </c>
       <c r="C507" t="inlineStr">
         <is>
@@ -16313,7 +16313,7 @@
         <v>45443</v>
       </c>
       <c r="B510">
-        <v>7383.1</v>
+        <v>10487.36</v>
       </c>
       <c r="C510" t="inlineStr">
         <is>
@@ -16336,7 +16336,7 @@
         <v>45443</v>
       </c>
       <c r="B511">
-        <v>6991.61</v>
+        <v>10385.9</v>
       </c>
       <c r="C511" t="inlineStr">
         <is>
@@ -16415,7 +16415,7 @@
         <v>45473</v>
       </c>
       <c r="B514">
-        <v>6283</v>
+        <v>10852.46</v>
       </c>
       <c r="C514" t="inlineStr">
         <is>
@@ -16514,7 +16514,7 @@
         <v>45473</v>
       </c>
       <c r="B517">
-        <v>6813.28</v>
+        <v>11768.4</v>
       </c>
       <c r="C517" t="inlineStr">
         <is>
@@ -16613,7 +16613,7 @@
         <v>45473</v>
       </c>
       <c r="B520">
-        <v>29320.69</v>
+        <v>50644.82</v>
       </c>
       <c r="C520" t="inlineStr">
         <is>
@@ -16712,7 +16712,7 @@
         <v>45473</v>
       </c>
       <c r="B523">
-        <v>31795.32</v>
+        <v>54919.19</v>
       </c>
       <c r="C523" t="inlineStr">
         <is>
@@ -16844,7 +16844,7 @@
         <v>45473</v>
       </c>
       <c r="B527">
-        <v>7363.99</v>
+        <v>10410.29</v>
       </c>
       <c r="C527" t="inlineStr">
         <is>
@@ -16867,7 +16867,7 @@
         <v>45473</v>
       </c>
       <c r="B528">
-        <v>6742.06</v>
+        <v>10045.47</v>
       </c>
       <c r="C528" t="inlineStr">
         <is>
@@ -16946,7 +16946,7 @@
         <v>45504</v>
       </c>
       <c r="B531">
-        <v>7150.09</v>
+        <v>12350.16</v>
       </c>
       <c r="C531" t="inlineStr">
         <is>
@@ -17045,7 +17045,7 @@
         <v>45504</v>
       </c>
       <c r="B534">
-        <v>7082.51</v>
+        <v>12233.43</v>
       </c>
       <c r="C534" t="inlineStr">
         <is>
@@ -17144,7 +17144,7 @@
         <v>45504</v>
       </c>
       <c r="B537">
-        <v>33367.1</v>
+        <v>57634.08</v>
       </c>
       <c r="C537" t="inlineStr">
         <is>
@@ -17243,7 +17243,7 @@
         <v>45504</v>
       </c>
       <c r="B540">
-        <v>33051.72</v>
+        <v>57089.34</v>
       </c>
       <c r="C540" t="inlineStr">
         <is>
@@ -17375,7 +17375,7 @@
         <v>45504</v>
       </c>
       <c r="B544">
-        <v>8271.969999999999</v>
+        <v>11738.68</v>
       </c>
       <c r="C544" t="inlineStr">
         <is>
@@ -17398,7 +17398,7 @@
         <v>45504</v>
       </c>
       <c r="B545">
-        <v>6839.06</v>
+        <v>10273</v>
       </c>
       <c r="C545" t="inlineStr">
         <is>
@@ -17477,7 +17477,7 @@
         <v>45535</v>
       </c>
       <c r="B548">
-        <v>7489.09</v>
+        <v>12935.71</v>
       </c>
       <c r="C548" t="inlineStr">
         <is>
@@ -17576,7 +17576,7 @@
         <v>45535</v>
       </c>
       <c r="B551">
-        <v>7190.55</v>
+        <v>12420.04</v>
       </c>
       <c r="C551" t="inlineStr">
         <is>
@@ -17675,7 +17675,7 @@
         <v>45535</v>
       </c>
       <c r="B554">
-        <v>34949.11</v>
+        <v>60366.64</v>
       </c>
       <c r="C554" t="inlineStr">
         <is>
@@ -17774,7 +17774,7 @@
         <v>45535</v>
       </c>
       <c r="B557">
-        <v>33555.91</v>
+        <v>57960.2</v>
       </c>
       <c r="C557" t="inlineStr">
         <is>
@@ -17873,7 +17873,7 @@
         <v>45535</v>
       </c>
       <c r="B560">
-        <v>8598.809999999999</v>
+        <v>12229.89</v>
       </c>
       <c r="C560" t="inlineStr">
         <is>
@@ -17896,7 +17896,7 @@
         <v>45535</v>
       </c>
       <c r="B561">
-        <v>7083.03</v>
+        <v>10569.36</v>
       </c>
       <c r="C561" t="inlineStr">
         <is>
@@ -17975,7 +17975,7 @@
         <v>45565</v>
       </c>
       <c r="B564">
-        <v>7650.84</v>
+        <v>13215.09</v>
       </c>
       <c r="C564" t="inlineStr">
         <is>
@@ -18074,7 +18074,7 @@
         <v>45565</v>
       </c>
       <c r="B567">
-        <v>7210.56</v>
+        <v>12454.61</v>
       </c>
       <c r="C567" t="inlineStr">
         <is>
@@ -18173,7 +18173,7 @@
         <v>45565</v>
       </c>
       <c r="B570">
-        <v>35703.93</v>
+        <v>61670.43</v>
       </c>
       <c r="C570" t="inlineStr">
         <is>
@@ -18272,7 +18272,7 @@
         <v>45565</v>
       </c>
       <c r="B573">
-        <v>33649.29</v>
+        <v>58121.51</v>
       </c>
       <c r="C573" t="inlineStr">
         <is>
@@ -18437,7 +18437,7 @@
         <v>45565</v>
       </c>
       <c r="B578">
-        <v>8428.34</v>
+        <v>12137.84</v>
       </c>
       <c r="C578" t="inlineStr">
         <is>
@@ -18460,7 +18460,7 @@
         <v>45565</v>
       </c>
       <c r="B579">
-        <v>7254.58</v>
+        <v>10750.61</v>
       </c>
       <c r="C579" t="inlineStr">
         <is>
@@ -18539,7 +18539,7 @@
         <v>45596</v>
       </c>
       <c r="B582">
-        <v>8516.65</v>
+        <v>14710.58</v>
       </c>
       <c r="C582" t="inlineStr">
         <is>
@@ -18638,7 +18638,7 @@
         <v>45596</v>
       </c>
       <c r="B585">
-        <v>8044.38</v>
+        <v>13894.84</v>
       </c>
       <c r="C585" t="inlineStr">
         <is>
@@ -18737,7 +18737,7 @@
         <v>45596</v>
       </c>
       <c r="B588">
-        <v>39744.38</v>
+        <v>68649.38</v>
       </c>
       <c r="C588" t="inlineStr">
         <is>
@@ -18836,7 +18836,7 @@
         <v>45596</v>
       </c>
       <c r="B591">
-        <v>37540.45</v>
+        <v>64842.59</v>
       </c>
       <c r="C591" t="inlineStr">
         <is>
@@ -19001,7 +19001,7 @@
         <v>45596</v>
       </c>
       <c r="B596">
-        <v>9383.65</v>
+        <v>13512.93</v>
       </c>
       <c r="C596" t="inlineStr">
         <is>
@@ -19024,7 +19024,7 @@
         <v>45596</v>
       </c>
       <c r="B597">
-        <v>7949.07</v>
+        <v>11849.38</v>
       </c>
       <c r="C597" t="inlineStr">
         <is>
@@ -19103,7 +19103,7 @@
         <v>45626</v>
       </c>
       <c r="B600">
-        <v>8213.68</v>
+        <v>14187.27</v>
       </c>
       <c r="C600" t="inlineStr">
         <is>
@@ -19202,7 +19202,7 @@
         <v>45626</v>
       </c>
       <c r="B603">
-        <v>8024.23</v>
+        <v>13860.03</v>
       </c>
       <c r="C603" t="inlineStr">
         <is>
@@ -19301,7 +19301,7 @@
         <v>45626</v>
       </c>
       <c r="B606">
-        <v>38330.53</v>
+        <v>66207.27</v>
       </c>
       <c r="C606" t="inlineStr">
         <is>
@@ -19400,7 +19400,7 @@
         <v>45626</v>
       </c>
       <c r="B609">
-        <v>37446.4</v>
+        <v>64680.14</v>
       </c>
       <c r="C609" t="inlineStr">
         <is>
@@ -19598,7 +19598,7 @@
         <v>45626</v>
       </c>
       <c r="B615">
-        <v>9260.07</v>
+        <v>13242.47</v>
       </c>
       <c r="C615" t="inlineStr">
         <is>
@@ -19621,7 +19621,7 @@
         <v>45626</v>
       </c>
       <c r="B616">
-        <v>8061.57</v>
+        <v>11952.11</v>
       </c>
       <c r="C616" t="inlineStr">
         <is>
@@ -19700,7 +19700,7 @@
         <v>45657</v>
       </c>
       <c r="B619">
-        <v>8356.209999999999</v>
+        <v>14433.45</v>
       </c>
       <c r="C619" t="inlineStr">
         <is>
@@ -19799,7 +19799,7 @@
         <v>45657</v>
       </c>
       <c r="B622">
-        <v>8589.4</v>
+        <v>14836.24</v>
       </c>
       <c r="C622" t="inlineStr">
         <is>
@@ -19898,7 +19898,7 @@
         <v>45657</v>
       </c>
       <c r="B625">
-        <v>38995.63</v>
+        <v>67356.09</v>
       </c>
       <c r="C625" t="inlineStr">
         <is>
@@ -19997,7 +19997,7 @@
         <v>45657</v>
       </c>
       <c r="B628">
-        <v>40083.89</v>
+        <v>69235.8</v>
       </c>
       <c r="C628" t="inlineStr">
         <is>
@@ -20162,7 +20162,7 @@
         <v>45657</v>
       </c>
       <c r="B633">
-        <v>9655.549999999999</v>
+        <v>13707.04</v>
       </c>
       <c r="C633" t="inlineStr">
         <is>
@@ -20185,7 +20185,7 @@
         <v>45657</v>
       </c>
       <c r="B634">
-        <v>8916.27</v>
+        <v>13080.82</v>
       </c>
       <c r="C634" t="inlineStr">
         <is>
@@ -20264,7 +20264,7 @@
         <v>45688</v>
       </c>
       <c r="B637">
-        <v>8637.76</v>
+        <v>14919.78</v>
       </c>
       <c r="C637" t="inlineStr">
         <is>
@@ -20363,7 +20363,7 @@
         <v>45688</v>
       </c>
       <c r="B640">
-        <v>9353.1</v>
+        <v>16155.36</v>
       </c>
       <c r="C640" t="inlineStr">
         <is>
@@ -20462,7 +20462,7 @@
         <v>45688</v>
       </c>
       <c r="B643">
-        <v>40309.57</v>
+        <v>69625.62</v>
       </c>
       <c r="C643" t="inlineStr">
         <is>
@@ -20561,7 +20561,7 @@
         <v>45688</v>
       </c>
       <c r="B646">
-        <v>43647.82</v>
+        <v>75391.67999999999</v>
       </c>
       <c r="C646" t="inlineStr">
         <is>
@@ -20693,7 +20693,7 @@
         <v>45688</v>
       </c>
       <c r="B650">
-        <v>10074.48</v>
+        <v>14262.48</v>
       </c>
       <c r="C650" t="inlineStr">
         <is>
@@ -20716,7 +20716,7 @@
         <v>45688</v>
       </c>
       <c r="B651">
-        <v>9659.950000000001</v>
+        <v>14194.79</v>
       </c>
       <c r="C651" t="inlineStr">
         <is>
@@ -20795,7 +20795,7 @@
         <v>45716</v>
       </c>
       <c r="B654">
-        <v>7883.3</v>
+        <v>13616.61</v>
       </c>
       <c r="C654" t="inlineStr">
         <is>
@@ -20894,7 +20894,7 @@
         <v>45716</v>
       </c>
       <c r="B657">
-        <v>9052.700000000001</v>
+        <v>15636.48</v>
       </c>
       <c r="C657" t="inlineStr">
         <is>
@@ -20993,7 +20993,7 @@
         <v>45716</v>
       </c>
       <c r="B660">
-        <v>36788.73</v>
+        <v>63544.17</v>
       </c>
       <c r="C660" t="inlineStr">
         <is>
@@ -21092,7 +21092,7 @@
         <v>45716</v>
       </c>
       <c r="B663">
-        <v>42245.93</v>
+        <v>72970.25</v>
       </c>
       <c r="C663" t="inlineStr">
         <is>
@@ -21257,7 +21257,7 @@
         <v>45716</v>
       </c>
       <c r="B668">
-        <v>9157.530000000001</v>
+        <v>12979.73</v>
       </c>
       <c r="C668" t="inlineStr">
         <is>
@@ -21280,7 +21280,7 @@
         <v>45716</v>
       </c>
       <c r="B669">
-        <v>9203.35</v>
+        <v>13592.53</v>
       </c>
       <c r="C669" t="inlineStr">
         <is>
@@ -21359,7 +21359,7 @@
         <v>45747</v>
       </c>
       <c r="B672">
-        <v>9303.49</v>
+        <v>16069.67</v>
       </c>
       <c r="C672" t="inlineStr">
         <is>
@@ -21458,7 +21458,7 @@
         <v>45747</v>
       </c>
       <c r="B675">
-        <v>10491.74</v>
+        <v>18122.1</v>
       </c>
       <c r="C675" t="inlineStr">
         <is>
@@ -21557,7 +21557,7 @@
         <v>45747</v>
       </c>
       <c r="B678">
-        <v>43416.3</v>
+        <v>74991.78</v>
       </c>
       <c r="C678" t="inlineStr">
         <is>
@@ -21656,7 +21656,7 @@
         <v>45747</v>
       </c>
       <c r="B681">
-        <v>48961.45</v>
+        <v>84569.78</v>
       </c>
       <c r="C681" t="inlineStr">
         <is>
@@ -21887,7 +21887,7 @@
         <v>45747</v>
       </c>
       <c r="B688">
-        <v>10720.02</v>
+        <v>15230.81</v>
       </c>
       <c r="C688" t="inlineStr">
         <is>
@@ -21910,7 +21910,7 @@
         <v>45747</v>
       </c>
       <c r="B689">
-        <v>10580.96</v>
+        <v>15667.86</v>
       </c>
       <c r="C689" t="inlineStr">
         <is>
@@ -21989,7 +21989,7 @@
         <v>45777</v>
       </c>
       <c r="B692">
-        <v>9701.389999999999</v>
+        <v>16756.94</v>
       </c>
       <c r="C692" t="inlineStr">
         <is>
@@ -22088,7 +22088,7 @@
         <v>45777</v>
       </c>
       <c r="B695">
-        <v>10304.42</v>
+        <v>17798.54</v>
       </c>
       <c r="C695" t="inlineStr">
         <is>
@@ -22187,7 +22187,7 @@
         <v>45777</v>
       </c>
       <c r="B698">
-        <v>45273.13</v>
+        <v>78199.05</v>
       </c>
       <c r="C698" t="inlineStr">
         <is>
@@ -22286,7 +22286,7 @@
         <v>45777</v>
       </c>
       <c r="B701">
-        <v>48087.27</v>
+        <v>83059.83</v>
       </c>
       <c r="C701" t="inlineStr">
         <is>
@@ -22484,7 +22484,7 @@
         <v>45777</v>
       </c>
       <c r="B707">
-        <v>11028.26</v>
+        <v>15731.96</v>
       </c>
       <c r="C707" t="inlineStr">
         <is>
@@ -22507,7 +22507,7 @@
         <v>45777</v>
       </c>
       <c r="B708">
-        <v>10385.88</v>
+        <v>15381.96</v>
       </c>
       <c r="C708" t="inlineStr">
         <is>
@@ -22586,7 +22586,7 @@
         <v>45808</v>
       </c>
       <c r="B711">
-        <v>10662.5</v>
+        <v>18417.04</v>
       </c>
       <c r="C711" t="inlineStr">
         <is>
@@ -22685,7 +22685,7 @@
         <v>45808</v>
       </c>
       <c r="B714">
-        <v>10109.51</v>
+        <v>17461.88</v>
       </c>
       <c r="C714" t="inlineStr">
         <is>
@@ -22784,7 +22784,7 @@
         <v>45808</v>
       </c>
       <c r="B717">
-        <v>49758.32</v>
+        <v>85946.17999999999</v>
       </c>
       <c r="C717" t="inlineStr">
         <is>
@@ -22883,7 +22883,7 @@
         <v>45808</v>
       </c>
       <c r="B720">
-        <v>47177.7</v>
+        <v>81488.75999999999</v>
       </c>
       <c r="C720" t="inlineStr">
         <is>
@@ -22982,7 +22982,7 @@
         <v>45808</v>
       </c>
       <c r="B723">
-        <v>12015.55</v>
+        <v>17185.25</v>
       </c>
       <c r="C723" t="inlineStr">
         <is>
@@ -23005,7 +23005,7 @@
         <v>45808</v>
       </c>
       <c r="B724">
-        <v>10402.89</v>
+        <v>15304.47</v>
       </c>
       <c r="C724" t="inlineStr">
         <is>
@@ -23084,7 +23084,7 @@
         <v>45838</v>
       </c>
       <c r="B727">
-        <v>10545.7</v>
+        <v>18215.3</v>
       </c>
       <c r="C727" t="inlineStr">
         <is>
@@ -23183,7 +23183,7 @@
         <v>45838</v>
       </c>
       <c r="B730">
-        <v>9857.83</v>
+        <v>17027.15</v>
       </c>
       <c r="C730" t="inlineStr">
         <is>
@@ -23282,7 +23282,7 @@
         <v>45838</v>
       </c>
       <c r="B733">
-        <v>49213.28</v>
+        <v>85004.75</v>
       </c>
       <c r="C733" t="inlineStr">
         <is>
@@ -23381,7 +23381,7 @@
         <v>45838</v>
       </c>
       <c r="B736">
-        <v>46003.19</v>
+        <v>79460.05</v>
       </c>
       <c r="C736" t="inlineStr">
         <is>
@@ -23447,7 +23447,7 @@
         <v>45838</v>
       </c>
       <c r="B738">
-        <v>12122.05</v>
+        <v>17235.12</v>
       </c>
       <c r="C738" t="inlineStr">
         <is>
@@ -23470,7 +23470,7 @@
         <v>45838</v>
       </c>
       <c r="B739">
-        <v>10230.84</v>
+        <v>15010.39</v>
       </c>
       <c r="C739" t="inlineStr">
         <is>
@@ -23549,7 +23549,7 @@
         <v>45869</v>
       </c>
       <c r="B742">
-        <v>10993.87</v>
+        <v>18989.42</v>
       </c>
       <c r="C742" t="inlineStr">
         <is>
@@ -23648,7 +23648,7 @@
         <v>45869</v>
       </c>
       <c r="B745">
-        <v>10834.67</v>
+        <v>18714.43</v>
       </c>
       <c r="C745" t="inlineStr">
         <is>
@@ -23747,7 +23747,7 @@
         <v>45869</v>
       </c>
       <c r="B748">
-        <v>51304.75</v>
+        <v>88617.28999999999</v>
       </c>
       <c r="C748" t="inlineStr">
         <is>
@@ -23846,7 +23846,7 @@
         <v>45869</v>
       </c>
       <c r="B751">
-        <v>50561.79</v>
+        <v>87334</v>
       </c>
       <c r="C751" t="inlineStr">
         <is>
@@ -24011,7 +24011,7 @@
         <v>45869</v>
       </c>
       <c r="B756">
-        <v>12970.21</v>
+        <v>18300.57</v>
       </c>
       <c r="C756" t="inlineStr">
         <is>
@@ -24034,7 +24034,7 @@
         <v>45869</v>
       </c>
       <c r="B757">
-        <v>11001.15</v>
+        <v>16254.33</v>
       </c>
       <c r="C757" t="inlineStr">
         <is>
@@ -24113,7 +24113,7 @@
         <v>45900</v>
       </c>
       <c r="B760">
-        <v>11251.81</v>
+        <v>19434.95</v>
       </c>
       <c r="C760" t="inlineStr">
         <is>
@@ -24212,7 +24212,7 @@
         <v>45900</v>
       </c>
       <c r="B763">
-        <v>11092.75</v>
+        <v>19160.2</v>
       </c>
       <c r="C763" t="inlineStr">
         <is>
@@ -24311,7 +24311,7 @@
         <v>45900</v>
       </c>
       <c r="B766">
-        <v>52508.46</v>
+        <v>90696.42999999999</v>
       </c>
       <c r="C766" t="inlineStr">
         <is>
@@ -24410,7 +24410,7 @@
         <v>45900</v>
       </c>
       <c r="B769">
-        <v>51766.16</v>
+        <v>89414.27</v>
       </c>
       <c r="C769" t="inlineStr">
         <is>
@@ -24575,7 +24575,7 @@
         <v>45900</v>
       </c>
       <c r="B774">
-        <v>13351.84</v>
+        <v>18807.26</v>
       </c>
       <c r="C774" t="inlineStr">
         <is>
@@ -24598,7 +24598,7 @@
         <v>45900</v>
       </c>
       <c r="B775">
-        <v>11978.03</v>
+        <v>17356.33</v>
       </c>
       <c r="C775" t="inlineStr">
         <is>
@@ -24677,7 +24677,7 @@
         <v>45930</v>
       </c>
       <c r="B778">
-        <v>10929.54</v>
+        <v>18878.29</v>
       </c>
       <c r="C778" t="inlineStr">
         <is>
@@ -24776,7 +24776,7 @@
         <v>45930</v>
       </c>
       <c r="B781">
-        <v>11270.1</v>
+        <v>19466.54</v>
       </c>
       <c r="C781" t="inlineStr">
         <is>
@@ -24875,7 +24875,7 @@
         <v>45930</v>
       </c>
       <c r="B784">
-        <v>51004.5</v>
+        <v>88098.69</v>
       </c>
       <c r="C784" t="inlineStr">
         <is>
@@ -24974,7 +24974,7 @@
         <v>45930</v>
       </c>
       <c r="B787">
-        <v>52593.81</v>
+        <v>90843.85000000001</v>
       </c>
       <c r="C787" t="inlineStr">
         <is>
@@ -25106,7 +25106,7 @@
         <v>45930</v>
       </c>
       <c r="B791">
-        <v>13229.38</v>
+        <v>18528.55</v>
       </c>
       <c r="C791" t="inlineStr">
         <is>
@@ -25129,7 +25129,7 @@
         <v>45930</v>
       </c>
       <c r="B792">
-        <v>12021.75</v>
+        <v>17486.04</v>
       </c>
       <c r="C792" t="inlineStr">
         <is>
@@ -25208,7 +25208,7 @@
         <v>45961</v>
       </c>
       <c r="B795">
-        <v>10995.32</v>
+        <v>18991.91</v>
       </c>
       <c r="C795" t="inlineStr">
         <is>
@@ -25307,7 +25307,7 @@
         <v>45961</v>
       </c>
       <c r="B798">
-        <v>11898.91</v>
+        <v>20552.67</v>
       </c>
       <c r="C798" t="inlineStr">
         <is>
@@ -25406,7 +25406,7 @@
         <v>45961</v>
       </c>
       <c r="B801">
-        <v>51311.48</v>
+        <v>88628.91</v>
       </c>
       <c r="C801" t="inlineStr">
         <is>
@@ -25505,7 +25505,7 @@
         <v>45961</v>
       </c>
       <c r="B804">
-        <v>55528.27</v>
+        <v>95912.46000000001</v>
       </c>
       <c r="C804" t="inlineStr">
         <is>
@@ -25670,7 +25670,7 @@
         <v>45961</v>
       </c>
       <c r="B809">
-        <v>13315.2</v>
+        <v>18646.27</v>
       </c>
       <c r="C809" t="inlineStr">
         <is>
@@ -25693,7 +25693,7 @@
         <v>45961</v>
       </c>
       <c r="B810">
-        <v>12458.13</v>
+        <v>18227.3</v>
       </c>
       <c r="C810" t="inlineStr">
         <is>
@@ -25772,7 +25772,7 @@
         <v>45991</v>
       </c>
       <c r="B813">
-        <v>10314.67</v>
+        <v>17816.24</v>
       </c>
       <c r="C813" t="inlineStr">
         <is>
@@ -25871,7 +25871,7 @@
         <v>45991</v>
       </c>
       <c r="B816">
-        <v>11862.51</v>
+        <v>20489.79</v>
       </c>
       <c r="C816" t="inlineStr">
         <is>
@@ -25970,7 +25970,7 @@
         <v>45991</v>
       </c>
       <c r="B819">
-        <v>48135.12</v>
+        <v>83142.47</v>
       </c>
       <c r="C819" t="inlineStr">
         <is>
@@ -26069,7 +26069,7 @@
         <v>45991</v>
       </c>
       <c r="B822">
-        <v>55358.38</v>
+        <v>95619.02</v>
       </c>
       <c r="C822" t="inlineStr">
         <is>
@@ -26201,7 +26201,7 @@
         <v>45991</v>
       </c>
       <c r="B826">
-        <v>13089.08</v>
+        <v>18090.13</v>
       </c>
       <c r="C826" t="inlineStr">
         <is>
@@ -26224,7 +26224,7 @@
         <v>45991</v>
       </c>
       <c r="B827">
-        <v>12202.17</v>
+        <v>17953.69</v>
       </c>
       <c r="C827" t="inlineStr">
         <is>
@@ -26303,7 +26303,7 @@
         <v>46022</v>
       </c>
       <c r="B830">
-        <v>10943.91</v>
+        <v>18903.11</v>
       </c>
       <c r="C830" t="inlineStr">
         <is>
@@ -26402,7 +26402,7 @@
         <v>46022</v>
       </c>
       <c r="B833">
-        <v>12549.88</v>
+        <v>21677.07</v>
       </c>
       <c r="C833" t="inlineStr">
         <is>
@@ -26501,7 +26501,7 @@
         <v>46022</v>
       </c>
       <c r="B836">
-        <v>51071.57</v>
+        <v>88214.52</v>
       </c>
       <c r="C836" t="inlineStr">
         <is>
@@ -26600,7 +26600,7 @@
         <v>46022</v>
       </c>
       <c r="B839">
-        <v>58566.11</v>
+        <v>101159.64</v>
       </c>
       <c r="C839" t="inlineStr">
         <is>
@@ -26798,7 +26798,7 @@
         <v>46022</v>
       </c>
       <c r="B845">
-        <v>14322.01</v>
+        <v>19628.14</v>
       </c>
       <c r="C845" t="inlineStr">
         <is>
@@ -26821,7 +26821,7 @@
         <v>46022</v>
       </c>
       <c r="B846">
-        <v>12663.23</v>
+        <v>18748.02</v>
       </c>
       <c r="C846" t="inlineStr">
         <is>

</xml_diff>